<commit_message>
Actualiza fecha y recompila informe 2026 en HTML, PDF y DOCX
</commit_message>
<xml_diff>
--- a/cursoPropedeuticoEstadistica/2026/relacionEstudiantesAprobados.xlsx
+++ b/cursoPropedeuticoEstadistica/2026/relacionEstudiantesAprobados.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oscardelatorretorres/Documents/GitHub/cursos/cursoPropedeuticoEstadistica/2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{531E2733-C8C0-EA4B-ACC3-82141167B5EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95803B75-30DF-7043-9706-5DBE0D59A873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="28200" xr2:uid="{433C1CA6-4746-314E-B0CC-0888E1E76245}"/>
   </bookViews>
   <sheets>
     <sheet name="Calificaciones" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -558,7 +558,7 @@
         <v>100</v>
       </c>
       <c r="D2" s="3">
-        <v>1.5384615384615385</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -572,7 +572,7 @@
         <v>100</v>
       </c>
       <c r="D3" s="3">
-        <v>5.9069230769230767</v>
+        <v>9.3369999999999997</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -586,7 +586,7 @@
         <v>100</v>
       </c>
       <c r="D4" s="3">
-        <v>6.6984615384615385</v>
+        <v>7.1807692307692301</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -642,7 +642,7 @@
         <v>100</v>
       </c>
       <c r="D8" s="3">
-        <v>7.287692307692307</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -684,7 +684,7 @@
         <v>100</v>
       </c>
       <c r="D11" s="3">
-        <v>7.8830769230769233</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -698,7 +698,7 @@
         <v>100</v>
       </c>
       <c r="D12" s="3">
-        <v>7.1807692307692301</v>
+        <v>8.2838461538461541</v>
       </c>
     </row>
   </sheetData>

</xml_diff>